<commit_message>
corrigindo o erro de não preencher o LI em ids do campo diferente
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Downloads\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780089D5-B0CB-40B0-8532-3DD4E465E540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5BA447-6BC8-4581-ACA3-85FD72E8F9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="154">
   <si>
     <t>Status</t>
   </si>
@@ -440,9 +440,6 @@
     <t>Modo</t>
   </si>
   <si>
-    <t>Simulado</t>
-  </si>
-  <si>
     <t>Criar Plano Manutenção Sem Estratégia - IP41 - Simular</t>
   </si>
   <si>
@@ -486,6 +483,9 @@
   </si>
   <si>
     <t>Nº equipamento: 10141343 | Texto Breve: testeO | TipoAtvMnt: 31 | Prioridade: 2 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
+  </si>
+  <si>
+    <t>simulado</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1476,7 @@
         <v>104</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>105</v>
@@ -1497,15 +1497,17 @@
       <c r="B3" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="19"/>
+      <c r="C3" s="19" t="s">
+        <v>153</v>
+      </c>
       <c r="D3" s="15" t="s">
         <v>105</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="13"/>
@@ -1517,15 +1519,17 @@
       <c r="B4" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="16"/>
+      <c r="C4" s="16" t="s">
+        <v>153</v>
+      </c>
       <c r="D4" s="16" t="s">
         <v>112</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="13"/>
@@ -1537,7 +1541,9 @@
       <c r="B5" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="15"/>
+      <c r="C5" s="15" t="s">
+        <v>153</v>
+      </c>
       <c r="D5" s="15" t="s">
         <v>107</v>
       </c>
@@ -1577,7 +1583,9 @@
       <c r="B7" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="15"/>
+      <c r="C7" s="15" t="s">
+        <v>153</v>
+      </c>
       <c r="D7" s="15" t="s">
         <v>107</v>
       </c>
@@ -1585,7 +1593,7 @@
         <v>131</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="13"/>
@@ -1595,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15" t="s">
@@ -1613,17 +1621,17 @@
         <v>1</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C9" s="15"/>
       <c r="D9" s="15" t="s">
         <v>109</v>
       </c>
       <c r="E9" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="F9" s="15" t="s">
         <v>141</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>142</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="13"/>
@@ -1633,17 +1641,17 @@
         <v>1</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15" t="s">
         <v>110</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="13"/>
@@ -1653,17 +1661,17 @@
         <v>1</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15" t="s">
         <v>111</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="13"/>

</xml_diff>

<commit_message>
Revert "Merge pull request #15 from Vitinhoorei/feat-diferentes-ids-LI"
This reverts commit d7b71c6db00ad2912b6d376d0fa353dabede7958, reversing
changes made to 60db362b9626ba2bc30a12dbb965f5d998a4dc80.
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Downloads\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA5BA447-6BC8-4581-ACA3-85FD72E8F9C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780089D5-B0CB-40B0-8532-3DD4E465E540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="413" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="154">
   <si>
     <t>Status</t>
   </si>
@@ -440,6 +440,9 @@
     <t>Modo</t>
   </si>
   <si>
+    <t>Simulado</t>
+  </si>
+  <si>
     <t>Criar Plano Manutenção Sem Estratégia - IP41 - Simular</t>
   </si>
   <si>
@@ -483,9 +486,6 @@
   </si>
   <si>
     <t>Nº equipamento: 10141343 | Texto Breve: testeO | TipoAtvMnt: 31 | Prioridade: 2 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
-  </si>
-  <si>
-    <t>simulado</t>
   </si>
 </sst>
 </file>
@@ -1476,7 +1476,7 @@
         <v>104</v>
       </c>
       <c r="C2" s="15" t="s">
-        <v>153</v>
+        <v>138</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>105</v>
@@ -1497,17 +1497,15 @@
       <c r="B3" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="19" t="s">
-        <v>153</v>
-      </c>
+      <c r="C3" s="19"/>
       <c r="D3" s="15" t="s">
         <v>105</v>
       </c>
       <c r="E3" s="15" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="F3" s="15" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="G3" s="15"/>
       <c r="H3" s="13"/>
@@ -1519,17 +1517,15 @@
       <c r="B4" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="16" t="s">
-        <v>153</v>
-      </c>
+      <c r="C4" s="16"/>
       <c r="D4" s="16" t="s">
         <v>112</v>
       </c>
       <c r="E4" s="16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F4" s="16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="G4" s="15"/>
       <c r="H4" s="13"/>
@@ -1541,9 +1537,7 @@
       <c r="B5" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="15" t="s">
-        <v>153</v>
-      </c>
+      <c r="C5" s="15"/>
       <c r="D5" s="15" t="s">
         <v>107</v>
       </c>
@@ -1583,9 +1577,7 @@
       <c r="B7" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="15" t="s">
-        <v>153</v>
-      </c>
+      <c r="C7" s="15"/>
       <c r="D7" s="15" t="s">
         <v>107</v>
       </c>
@@ -1593,7 +1585,7 @@
         <v>131</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="G7" s="15"/>
       <c r="H7" s="13"/>
@@ -1603,7 +1595,7 @@
         <v>1</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15" t="s">
@@ -1621,17 +1613,17 @@
         <v>1</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C9" s="15"/>
       <c r="D9" s="15" t="s">
         <v>109</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="G9" s="15"/>
       <c r="H9" s="13"/>
@@ -1641,17 +1633,17 @@
         <v>1</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C10" s="15"/>
       <c r="D10" s="15" t="s">
         <v>110</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F10" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G10" s="15"/>
       <c r="H10" s="13"/>
@@ -1661,17 +1653,17 @@
         <v>1</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C11" s="15"/>
       <c r="D11" s="15" t="s">
         <v>111</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F11" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G11" s="15"/>
       <c r="H11" s="13"/>

</xml_diff>

<commit_message>
Tentando arrumar para apontar horas
</commit_message>
<xml_diff>
--- a/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
+++ b/data/input/Cenários de Testes Unitários e Parciais - PM-Manutenção (1).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\juscelinob\Downloads\automated-integrated-tests\data\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{780089D5-B0CB-40B0-8532-3DD4E465E540}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7642E939-D70C-4D39-BE7D-1FF2D64763B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="409" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="416" uniqueCount="156">
   <si>
     <t>Status</t>
   </si>
@@ -486,13 +486,19 @@
   </si>
   <si>
     <t>Nº equipamento: 10141343 | Texto Breve: testeO | TipoAtvMnt: 31 | Prioridade: 2 | Criar Nota: x | Notificador: teste | Prioridade da Nota: 1 | Ramal: 1111 | Trabalho: 1 | Nº Colaboradores: 1</t>
+  </si>
+  <si>
+    <t>simulado</t>
+  </si>
+  <si>
+    <t>executar</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -642,6 +648,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1046,7 +1060,7 @@
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="33" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1087,6 +1101,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20% - Ênfase1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1497,7 +1514,9 @@
       <c r="B3" s="15" t="s">
         <v>125</v>
       </c>
-      <c r="C3" s="19"/>
+      <c r="C3" s="19" t="s">
+        <v>154</v>
+      </c>
       <c r="D3" s="15" t="s">
         <v>105</v>
       </c>
@@ -1517,7 +1536,9 @@
       <c r="B4" s="16" t="s">
         <v>128</v>
       </c>
-      <c r="C4" s="16"/>
+      <c r="C4" s="16" t="s">
+        <v>155</v>
+      </c>
       <c r="D4" s="16" t="s">
         <v>112</v>
       </c>
@@ -1537,7 +1558,9 @@
       <c r="B5" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="C5" s="15"/>
+      <c r="C5" s="15" t="s">
+        <v>155</v>
+      </c>
       <c r="D5" s="15" t="s">
         <v>107</v>
       </c>
@@ -1557,7 +1580,9 @@
       <c r="B6" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="C6" s="15"/>
+      <c r="C6" s="15" t="s">
+        <v>155</v>
+      </c>
       <c r="D6" s="15" t="s">
         <v>107</v>
       </c>
@@ -1577,7 +1602,9 @@
       <c r="B7" s="15" t="s">
         <v>136</v>
       </c>
-      <c r="C7" s="15"/>
+      <c r="C7" s="15" t="s">
+        <v>154</v>
+      </c>
       <c r="D7" s="15" t="s">
         <v>107</v>
       </c>
@@ -1597,7 +1624,9 @@
       <c r="B8" s="15" t="s">
         <v>140</v>
       </c>
-      <c r="C8" s="15"/>
+      <c r="C8" s="15" t="s">
+        <v>154</v>
+      </c>
       <c r="D8" s="15" t="s">
         <v>108</v>
       </c>
@@ -1615,7 +1644,9 @@
       <c r="B9" s="15" t="s">
         <v>146</v>
       </c>
-      <c r="C9" s="15"/>
+      <c r="C9" s="15" t="s">
+        <v>154</v>
+      </c>
       <c r="D9" s="15" t="s">
         <v>109</v>
       </c>
@@ -1662,7 +1693,7 @@
       <c r="E11" s="15" t="s">
         <v>145</v>
       </c>
-      <c r="F11" s="16" t="s">
+      <c r="F11" s="20" t="s">
         <v>147</v>
       </c>
       <c r="G11" s="15"/>

</xml_diff>